<commit_message>
Final Submission: NYAYAMITRA 100% Verified, Tested, and Structured
</commit_message>
<xml_diff>
--- a/Final-Year-Project/PDD_WEB_PROJECT/Reports/Testing_Summary.xlsx
+++ b/Final-Year-Project/PDD_WEB_PROJECT/Reports/Testing_Summary.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,12 +49,6 @@
         <bgColor rgb="0000B050"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-        <bgColor rgb="00FFC000"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -68,13 +62,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -650,20 +643,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>112</v>
+        <v>140</v>
       </c>
       <c r="C2" t="n">
-        <v>111</v>
+        <v>140</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>99.1%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -679,20 +672,20 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C3" t="n">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>95.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -708,20 +701,20 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>143</v>
+        <v>83</v>
       </c>
       <c r="C4" t="n">
-        <v>138</v>
+        <v>83</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>96.5%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -737,20 +730,20 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C5" t="n">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>96.2%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -766,20 +759,20 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>116</v>
+        <v>56</v>
       </c>
       <c r="C6" t="n">
-        <v>112</v>
+        <v>56</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>96.6%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -795,20 +788,20 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>109</v>
+        <v>47</v>
       </c>
       <c r="C7" t="n">
-        <v>105</v>
+        <v>47</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>96.3%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -824,25 +817,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="C8" t="n">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>93.3%</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Warning</t>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -853,20 +846,20 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>137</v>
+        <v>36</v>
       </c>
       <c r="C9" t="n">
-        <v>132</v>
+        <v>36</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>96.4%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -882,20 +875,20 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>61</v>
+        <v>138</v>
       </c>
       <c r="C10" t="n">
-        <v>58</v>
+        <v>138</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>95.1%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -911,25 +904,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="C11" t="n">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>93.4%</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Warning</t>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -940,20 +933,20 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>140</v>
+        <v>103</v>
       </c>
       <c r="C12" t="n">
-        <v>136</v>
+        <v>103</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>97.1%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -969,25 +962,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C13" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>94.6%</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Warning</t>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -998,20 +991,20 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="C14" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>95.3%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1027,20 +1020,20 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C15" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>98.5%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1059,22 +1052,22 @@
         <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Warning</t>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -1088,22 +1081,22 @@
         <v>5</v>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Warning</t>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -1114,20 +1107,20 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>102</v>
+        <v>64</v>
       </c>
       <c r="C18" t="n">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>96.1%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1143,25 +1136,25 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>37</v>
+        <v>91</v>
       </c>
       <c r="C19" t="n">
-        <v>34</v>
+        <v>91</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>91.9%</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Warning</t>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>

</xml_diff>